<commit_message>
Who owes me card names each customer; tracker summary tab renamed
- Sample card lists Bayou View Church $425 (41 days, call first), Pine Ave.
  Office $240, Live Oak Lane $900 (not billed), total $1,565, quote waiting.
- Free tracker: 'Who Owes Me' tab (totals only) renamed 'What I'm Owed';
  Start Here explains how to see names on the Jobs tab. Recalculated, 0 errors.
- Service card: 'A list of who owes you and how much, with totals'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UT1crtYU78jrkCbYZTsq92
</commit_message>
<xml_diff>
--- a/downloads/StoneRiver-Job-and-Invoice-Tracker.xlsx
+++ b/downloads/StoneRiver-Job-and-Invoice-Tracker.xlsx
@@ -10,7 +10,7 @@
   <sheets>
     <sheet name="Start Here" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Jobs" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Who Owes Me" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="What I'm Owed" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Jobs!$1:$1</definedName>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">JOB &amp; INVOICE TRACKER</t>
   </si>
@@ -48,7 +48,10 @@
     <t xml:space="preserve">4.  When you send the bill, type the Invoice date. When money comes in, type it in Paid ($).</t>
   </si>
   <si>
-    <t xml:space="preserve">5.  Open the Who Owes Me tab any time to see what's still out and how long it's been.</t>
+    <t xml:space="preserve">5.  To see WHO owes you: on the Jobs tab, sort by Balance or Days since invoice (largest first). Red rows are over 30 days.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.  The What I'm Owed tab adds it all up: total owed, how much is over 30 days, jobs not billed yet.</t>
   </si>
   <si>
     <t xml:space="preserve">What to type in</t>
@@ -126,10 +129,10 @@
     <t xml:space="preserve">EXAMPLE ROW – delete or type over it</t>
   </si>
   <si>
-    <t xml:space="preserve">WHO OWES ME</t>
+    <t xml:space="preserve">WHAT I'M OWED</t>
   </si>
   <si>
-    <t xml:space="preserve">Updates itself from the Jobs tab.</t>
+    <t xml:space="preserve">Totals that update themselves from the Jobs tab. For names, see the Jobs tab (red rows = over 30 days).</t>
   </si>
   <si>
     <t xml:space="preserve">Total billed (all jobs)</t>
@@ -746,7 +749,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:B21"/>
+  <dimension ref="B2:B22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -788,58 +791,63 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="4" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="3" t="s">
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="4" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -876,40 +884,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -920,16 +928,16 @@
         <v>46296</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G2" s="9" t="n">
         <v>160</v>
@@ -949,7 +957,7 @@
         <v>16</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4972,17 +4980,17 @@
   <sheetData>
     <row r="2" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" s="21" t="n">
         <f aca="false">SUM(Jobs!$G$2:$G$201)</f>
@@ -4991,7 +4999,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="21" t="n">
         <f aca="false">SUM(Jobs!$H$2:$H$201)</f>
@@ -5000,7 +5008,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" s="21" t="n">
         <f aca="false">SUMIF(Jobs!$I$2:$I$201,"&gt;0")</f>
@@ -5009,7 +5017,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C8" s="21" t="n">
         <f aca="false">SUMIFS(Jobs!$I$2:$I$201,Jobs!$I$2:$I$201,"&gt;0",Jobs!$K$2:$K$201,"&gt;30")</f>
@@ -5018,7 +5026,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="20" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" s="23" t="n">
         <f aca="false">COUNTIFS(Jobs!$I$2:$I$201,"&gt;0",Jobs!$J$2:$J$201,"&lt;&gt;")</f>
@@ -5027,7 +5035,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" s="23" t="n">
         <f aca="false">COUNTIF(Jobs!$F$2:$F$201,"Done")</f>
@@ -5036,7 +5044,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">COUNTIF(Jobs!$F$2:$F$201,"Quoted")</f>
@@ -5045,12 +5053,12 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="24" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Switch business phone to local 228 number (228) 901-3370
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GvEkDADL33wEAMDfKSvTqx
</commit_message>
<xml_diff>
--- a/downloads/StoneRiver-Job-and-Invoice-Tracker.xlsx
+++ b/downloads/StoneRiver-Job-and-Invoice-Tracker.xlsx
@@ -648,13 +648,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:B23"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="26" min="1" max="1"/>
     <col width="95" customWidth="1" style="26" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26.8" customHeight="1" s="27">
       <c r="B2" s="28" t="inlineStr">
         <is>
@@ -669,6 +670,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="16.15" customHeight="1" s="27">
       <c r="B5" s="30" t="inlineStr">
         <is>
@@ -779,7 +781,7 @@
     <row r="22" ht="26.85" customHeight="1" s="27">
       <c r="B22" s="31" t="inlineStr">
         <is>
-          <t>Marcus Johnson · (225) 317-6653 · marcus@stonerivercoast.com</t>
+          <t>Marcus Johnson · (228) 901-3370 · marcus@stonerivercoast.com</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:C15"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="26" min="1" max="1"/>
@@ -4949,6 +4951,7 @@
     <col width="18" customWidth="1" style="26" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24.45" customHeight="1" s="27">
       <c r="B2" s="46" t="inlineStr">
         <is>
@@ -4963,6 +4966,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="27">
       <c r="B5" s="48" t="inlineStr">
         <is>
@@ -5040,6 +5044,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="23.85" customHeight="1" s="27">
       <c r="B13" s="52" t="inlineStr">
         <is>
@@ -5047,10 +5052,11 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="27">
       <c r="B15" s="53" t="inlineStr">
         <is>
-          <t>Want it set up with your real jobs? Free checkup: stonerivercoast.com/#free · Marcus, (225) 317-6653</t>
+          <t>Want it set up with your real jobs? Free checkup: stonerivercoast.com/#free · Marcus, (228) 901-3370</t>
         </is>
       </c>
     </row>

</xml_diff>